<commit_message>
feat: add 4th sample_image_questions.xlsx template covering question and option image edge cases and verify 100% full coverage
</commit_message>
<xml_diff>
--- a/excels/sample_awa_questions.xlsx
+++ b/excels/sample_awa_questions.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -517,6 +517,11 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Question Images</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Answer Images</t>
         </is>
       </c>
     </row>
@@ -559,6 +564,7 @@
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -599,6 +605,7 @@
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -639,6 +646,7 @@
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -679,6 +687,7 @@
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -719,6 +728,7 @@
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -759,6 +769,7 @@
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -799,6 +810,7 @@
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -839,6 +851,7 @@
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -879,6 +892,7 @@
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -919,6 +933,7 @@
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>